<commit_message>
Reviewed everyting except for chapter 7
</commit_message>
<xml_diff>
--- a/chapter7_config.xlsx
+++ b/chapter7_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JonathanVandenBerk\Desktop\Cursor_GIT\Magics_cursor_AI_workspace\Projects\VISION_test_plan_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED96583-1573-4C78-9DFC-6DC2B944C9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050C169D-8850-4E08-B90C-588726F6B284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25770" yWindow="720" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -1850,9 +1850,6 @@
     <t>Fixed to 10b for all tests</t>
   </si>
   <si>
-    <t>Features are included as functional test: Exposure time, sub-sampling, X-Y mirroring, ADC resolution</t>
-  </si>
-  <si>
     <t>M3802</t>
   </si>
   <si>
@@ -1869,6 +1866,9 @@
   </si>
   <si>
     <t>Only tested at speed during characterization (FHD30 mode), production testing uses FHD10, HD40 and VGA50 mode what is at half of the max speed</t>
+  </si>
+  <si>
+    <t>Features are tested during characterization: Exposure time, sub-sampling, X-Y mirroring, ADC resolution</t>
   </si>
 </sst>
 </file>
@@ -4640,15 +4640,15 @@
         <v>35</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="K28" s="9"/>
       <c r="L28" s="9"/>
       <c r="M28" s="9" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
@@ -4673,15 +4673,15 @@
         <v>35</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="9"/>
       <c r="M29" s="9" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
@@ -4977,10 +4977,10 @@
         <v>595</v>
       </c>
       <c r="I41" s="24" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="J41" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K41" s="23"/>
       <c r="L41" s="23"/>
@@ -5006,10 +5006,10 @@
         <v>594</v>
       </c>
       <c r="I42" s="24" t="s">
+        <v>607</v>
+      </c>
+      <c r="J42" s="24" t="s">
         <v>608</v>
-      </c>
-      <c r="J42" s="24" t="s">
-        <v>609</v>
       </c>
       <c r="K42" s="23"/>
       <c r="L42" s="23"/>
@@ -5038,7 +5038,7 @@
         <v>596</v>
       </c>
       <c r="J43" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K43" s="23"/>
       <c r="L43" s="23"/>
@@ -5067,7 +5067,7 @@
         <v>597</v>
       </c>
       <c r="J44" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K44" s="23"/>
       <c r="L44" s="23"/>
@@ -5096,7 +5096,7 @@
         <v>598</v>
       </c>
       <c r="J45" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K45" s="23"/>
       <c r="L45" s="23"/>
@@ -5125,7 +5125,7 @@
         <v>600</v>
       </c>
       <c r="J46" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K46" s="23"/>
       <c r="L46" s="23"/>
@@ -5154,7 +5154,7 @@
         <v>601</v>
       </c>
       <c r="J47" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K47" s="23"/>
       <c r="L47" s="23"/>
@@ -5183,7 +5183,7 @@
         <v>602</v>
       </c>
       <c r="J48" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K48" s="23"/>
       <c r="L48" s="23"/>
@@ -5214,7 +5214,7 @@
         <v>603</v>
       </c>
       <c r="J49" s="24" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K49" s="23"/>
       <c r="L49" s="23"/>
@@ -5267,7 +5267,7 @@
       <c r="K51" s="23"/>
       <c r="L51" s="23"/>
       <c r="M51" s="24" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>